<commit_message>
feat(3_boletas): recibos de medidor pagado + boletas corregidas del 01/08
recibos_medidor_pagado.py emite la constancia serie MP- y generar_corregidos.py
reimprime la boleta cuando un reclamo prospera (los .docx generados quedan
fuera de git). Suma el README del modulo y formato_recibo_medidor_pagado.html.

Entran tambien los 26 reclamos del 01/08 con su CONSOLIDADO.md, las lecturas
de agosto de 2_planilla y el registro del operario del ciclo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3_boletas/enriquecimiento/inputs/config_mes.xlsx
+++ b/3_boletas/enriquecimiento/inputs/config_mes.xlsx
@@ -658,29 +658,29 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>11/05/2026 al 10/06/2026</t>
+          <t>11/06/2026 al 10/07/2026</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>46208</v>
+        <v>46236</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>46206</v>
+        <v>46230</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>46152</v>
+        <v>46183</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>46183</v>
+        <v>46213</v>
       </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>04-05/07/2026</t>
+          <t>01-02/08/2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4-8pm</t>
+          <t>4-6pm</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>17471</v>
+        <v>17970</v>
       </c>
     </row>
   </sheetData>

</xml_diff>